<commit_message>
Added code to icl-hbv to have "no treatment" scenario, because current treatment status quo scenario has a treatment initiation rate that leads to ~70% treatment coverage by 2100. Also added preliminary scripts to plot graphs
</commit_message>
<xml_diff>
--- a/resources/ListOfCountryRegions.xlsx
+++ b/resources/ListOfCountryRegions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/mpickles_ic_ac_uk/Documents/Dropbox_copy/Hepatits B/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mpickles\Documents\Hepatitis_B\icl-hbv\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="386" documentId="8_{0BB9CF4B-82BA-4252-8512-D634B8358AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AEC7B7F-5590-4D1E-B083-9FCD42F02916}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642049B3-0A73-4C0D-BEC3-D3E2F20885DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{BC12BF35-FAF3-49E6-A2B4-C68B7322CEB3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{BC12BF35-FAF3-49E6-A2B4-C68B7322CEB3}"/>
   </bookViews>
   <sheets>
     <sheet name="GBD" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">WHO_regions!$A$1:$D$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">WorldBankIncomeGroups!$A$1:$F$219</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2854" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2859" uniqueCount="585">
   <si>
     <t>Togo</t>
   </si>
@@ -1796,6 +1797,12 @@
   </si>
   <si>
     <t>Southeast Asia, east Asia, and Oceania</t>
+  </si>
+  <si>
+    <t>Venezuela, RB, classified as an upper-middle income country until FY21, has been unclassified since then due to the unavailability of data (https://datahelpdesk.worldbank.org/knowledgebase/articles/906519-world-bank-country-and-lending-groups). I am using the 2021 classification</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ethiopia is currently in a temporary status of unclassification for FY26 (https://datahelpdesk.worldbank.org/knowledgebase/articles/906519-world-bank-country-and-lending-groups) - so I am using the 2025 classification. See Dropbox/HepB/Data/CountryClassification/WB_Historical_classification_2026_03_10.xlsx</t>
   </si>
 </sst>
 </file>
@@ -1924,10 +1931,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8044,13 +8047,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{215C42F6-EF60-4963-88C0-BF91415F3AE6}">
-  <dimension ref="A1:E219"/>
+  <dimension ref="A1:F219"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="40.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>403</v>
       </c>
@@ -8066,8 +8069,11 @@
       <c r="E1" s="6" t="s">
         <v>534</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F1" s="6" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>56</v>
       </c>
@@ -8084,7 +8090,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>305</v>
       </c>
@@ -8101,7 +8107,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>261</v>
       </c>
@@ -8118,7 +8124,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>425</v>
       </c>
@@ -8133,7 +8139,7 @@
       </c>
       <c r="E5" s="4"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>429</v>
       </c>
@@ -8148,7 +8154,7 @@
       </c>
       <c r="E6" s="4"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>346</v>
       </c>
@@ -8165,7 +8171,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>95</v>
       </c>
@@ -8182,7 +8188,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>166</v>
       </c>
@@ -8199,7 +8205,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>348</v>
       </c>
@@ -8216,7 +8222,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>434</v>
       </c>
@@ -8231,7 +8237,7 @@
       </c>
       <c r="E11" s="4"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>168</v>
       </c>
@@ -8246,7 +8252,7 @@
       </c>
       <c r="E12" s="4"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>83</v>
       </c>
@@ -8261,7 +8267,7 @@
       </c>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>376</v>
       </c>
@@ -8278,7 +8284,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>436</v>
       </c>
@@ -8293,7 +8299,7 @@
       </c>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>214</v>
       </c>
@@ -9098,7 +9104,7 @@
       </c>
       <c r="E64" s="4"/>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="4" t="s">
         <v>146</v>
       </c>
@@ -9115,7 +9121,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="4" t="s">
         <v>241</v>
       </c>
@@ -9125,12 +9131,17 @@
       <c r="C66" s="7" t="s">
         <v>431</v>
       </c>
-      <c r="D66" s="8"/>
+      <c r="D66" s="7" t="s">
+        <v>420</v>
+      </c>
       <c r="E66" s="7" t="s">
         <v>421</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F66" s="7" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="4" t="s">
         <v>457</v>
       </c>
@@ -9145,7 +9156,7 @@
       </c>
       <c r="E67" s="4"/>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="4" t="s">
         <v>190</v>
       </c>
@@ -9162,7 +9173,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="4" t="s">
         <v>123</v>
       </c>
@@ -9177,7 +9188,7 @@
       </c>
       <c r="E69" s="4"/>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="4" t="s">
         <v>77</v>
       </c>
@@ -9192,7 +9203,7 @@
       </c>
       <c r="E70" s="4"/>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="4" t="s">
         <v>459</v>
       </c>
@@ -9207,7 +9218,7 @@
       </c>
       <c r="E71" s="4"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="4" t="s">
         <v>204</v>
       </c>
@@ -9224,7 +9235,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="4" t="s">
         <v>461</v>
       </c>
@@ -9241,7 +9252,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="4" t="s">
         <v>293</v>
       </c>
@@ -9258,7 +9269,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="4" t="s">
         <v>162</v>
       </c>
@@ -9273,7 +9284,7 @@
       </c>
       <c r="E75" s="4"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="4" t="s">
         <v>134</v>
       </c>
@@ -9290,7 +9301,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="4" t="s">
         <v>462</v>
       </c>
@@ -9305,7 +9316,7 @@
       </c>
       <c r="E77" s="4"/>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" s="4" t="s">
         <v>464</v>
       </c>
@@ -9320,7 +9331,7 @@
       </c>
       <c r="E78" s="4"/>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" s="4" t="s">
         <v>466</v>
       </c>
@@ -9335,7 +9346,7 @@
       </c>
       <c r="E79" s="4"/>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="4" t="s">
         <v>281</v>
       </c>
@@ -11444,7 +11455,7 @@
       </c>
       <c r="E208" s="4"/>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A209" s="4" t="s">
         <v>527</v>
       </c>
@@ -11459,7 +11470,7 @@
       </c>
       <c r="E209" s="4"/>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A210" s="4" t="s">
         <v>101</v>
       </c>
@@ -11476,7 +11487,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A211" s="4" t="s">
         <v>1</v>
       </c>
@@ -11493,7 +11504,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A212" s="4" t="s">
         <v>360</v>
       </c>
@@ -11510,7 +11521,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A213" s="4" t="s">
         <v>528</v>
       </c>
@@ -11520,12 +11531,17 @@
       <c r="C213" s="7" t="s">
         <v>433</v>
       </c>
-      <c r="D213" s="4"/>
+      <c r="D213" s="7" t="s">
+        <v>423</v>
+      </c>
       <c r="E213" s="7" t="s">
         <v>424</v>
       </c>
-    </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F213" s="7" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A214" s="4" t="s">
         <v>529</v>
       </c>
@@ -11542,7 +11558,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A215" s="4" t="s">
         <v>530</v>
       </c>
@@ -11557,7 +11573,7 @@
       </c>
       <c r="E215" s="4"/>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A216" s="4" t="s">
         <v>532</v>
       </c>
@@ -11572,7 +11588,7 @@
       </c>
       <c r="E216" s="4"/>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A217" s="4" t="s">
         <v>533</v>
       </c>
@@ -11589,7 +11605,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A218" s="4" t="s">
         <v>267</v>
       </c>
@@ -11606,7 +11622,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A219" s="4" t="s">
         <v>243</v>
       </c>

</xml_diff>